<commit_message>
Fix RTP SEO import sheet: use store import-template layout
The first sheet was built from the product EXPORT layout (37 cols, extra
columns + different tail order), which the importer rejected (success:0 /
failure:14). Rebuild in the import TEMPLATE's exact 34-column order, Product ID
as int, type:3d pointer + price + media preserved. Generator now takes the
template + export + SEO JSON so it stays correct for the FR/IT/ES migration.
</commit_message>
<xml_diff>
--- a/ready-to-play/seo/rtp-SEO-update-EN.xlsx
+++ b/ready-to-play/seo/rtp-SEO-update-EN.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AK16"/>
+  <dimension ref="A1:AH16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -569,37 +569,22 @@
       </c>
       <c r="AE1" t="inlineStr">
         <is>
+          <t>Variant Note 1</t>
+        </is>
+      </c>
+      <c r="AF1" t="inlineStr">
+        <is>
+          <t>Variant Note 2</t>
+        </is>
+      </c>
+      <c r="AG1" t="inlineStr">
+        <is>
           <t>Inventory</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
-        <is>
-          <t>Product Sales</t>
-        </is>
-      </c>
-      <c r="AG1" t="inlineStr">
+      <c r="AH1" t="inlineStr">
         <is>
           <t>*Media</t>
-        </is>
-      </c>
-      <c r="AH1" t="inlineStr">
-        <is>
-          <t>Product image description (ALT)</t>
-        </is>
-      </c>
-      <c r="AI1" t="inlineStr">
-        <is>
-          <t>Variant URL</t>
-        </is>
-      </c>
-      <c r="AJ1" t="inlineStr">
-        <is>
-          <t>Variant Note 1</t>
-        </is>
-      </c>
-      <c r="AK1" t="inlineStr">
-        <is>
-          <t>Variant Note 2</t>
         </is>
       </c>
     </row>
@@ -621,12 +606,13 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>For multi-style products: The first line of the same product should be filled with 'M' (product main body), and the non-first line should be filled with 'P' (sub-style).For single-style product: Fill in 'S'</t>
+          <t>For multi-style products: The first line of the same product should be filled with 'M' (product main body), and the non-first line should be filled with 'P' (sub-style)
+For single-style product: Fill in "S"</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Maximum 255 characters for product subtitle</t>
+          <t>Maximum 60 characters for product subtitle</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -646,17 +632,17 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Maximum 250 characters</t>
+          <t>maximum 250 characters</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>maximum 2048 characters for SEO description</t>
+          <t>maximum 511 characters for SEO description</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>maximum 2048 characters</t>
+          <t>maximum 20 characters</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -756,54 +742,34 @@
       </c>
       <c r="AE2" t="inlineStr">
         <is>
+          <t>maximum 512 characters</t>
+        </is>
+      </c>
+      <c r="AF2" t="inlineStr">
+        <is>
+          <t>maximum 512 characters</t>
+        </is>
+      </c>
+      <c r="AG2" t="inlineStr">
+        <is>
           <t>maximum 7 digits</t>
         </is>
       </c>
-      <c r="AF2" t="inlineStr">
-        <is>
-          <t>The actual sales volume of the product (invalid when importing)</t>
-        </is>
-      </c>
-      <c r="AG2" t="inlineStr">
+      <c r="AH2" t="inlineStr">
         <is>
           <t>1. At least one image URL must be filled in for the rows with the product attribute 'M' (product main body) and 'S' (single-style product). Multiple URLs can be filled in and separated by commas. The first URL filled in by default is the product main image URL
 2.The rows with the product attribute 'P' (sub-style) only support one URL, and if multiple URLs are filled in, the first one will be imported by default. If left blank, no image is required by default
 3.If some sub-styles of the same product upload images, the remaining styles also need to upload images, otherwise the main product image will be filled in by default.</t>
         </is>
       </c>
-      <c r="AH2" t="inlineStr">
-        <is>
-          <t>Each image ALT will be separated by | and null values will not be hidden.</t>
-        </is>
-      </c>
-      <c r="AI2" t="inlineStr">
-        <is>
-          <t>The variant URL can be appended to the product link to automatically select a specific SKU, which is the content following the product handle in the SEO URL, such as: store domain/products/SEO URL Handle?variant_sku_code=xxxx (this field is invalid when importing products).</t>
-        </is>
-      </c>
-      <c r="AJ2" t="inlineStr">
-        <is>
-          <t>Maximum 512 characters</t>
-        </is>
-      </c>
-      <c r="AK2" t="inlineStr">
-        <is>
-          <t>Maximum 512 characters</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>10299141</v>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>2026-06-23T13:53:05-05:00</t>
-        </is>
+        <v>10294535</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>The Fracture - Full Kit</t>
+          <t>The Apex</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -814,38 +780,38 @@
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Ready-to-Play Full Kit — Jersey + Shorts</t>
+          <t>Ready-to-Play — Customize in seconds</t>
         </is>
       </c>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Angular shards that break the standard. Complete matchday kit — jersey + matching shorts, fully customizable with your name and number.</t>
+          <t>Bold angular shoulder panels in navy &amp; volt by default — fully recolorable. Add your name and number and play this week.</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>{"type":"3d","mudel":"configId=mamuto316759&amp;suitName=mamuto3","activity":"","productId":"16759"}</t>
+          <t>{"type":"3d","mudel":"configId=mamuto316578&amp;suitName=mamuto3","activity":"","productId":"16578"}</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>The Fracture Full Kit — Jersey + Shorts | MOMUTO</t>
+          <t>The Apex — Custom Football Jersey | MOMUTO</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>The Fracture full kit — custom jersey + matching shorts in your colors, name and number, previewed live. Ready-to-Play, no minimum order.</t>
+          <t>Customize The Apex football jersey — your colors, name and number, previewed live. Ready-to-Play from €19.70. No minimum order, every order purchase-protected.</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>the-fracture-full-kit</t>
+          <t>the-apex</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>custom football full kit, the fracture jersey, momuto, ready to play kit, personalized soccer jersey, modern football kit, jersey and shorts, full football kit</t>
+          <t>custom football jersey, the apex jersey, momuto, ready to play kit, personalized soccer jersey, custom team kit</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -860,7 +826,7 @@
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>669902430384160770</t>
+          <t>667755455610748930</t>
         </is>
       </c>
       <c r="Q3" t="n">
@@ -881,44 +847,34 @@
       <c r="X3" t="inlineStr"/>
       <c r="Y3" t="inlineStr"/>
       <c r="Z3" t="n">
-        <v>51.1</v>
+        <v>35</v>
       </c>
       <c r="AA3" t="n">
         <v>0</v>
       </c>
       <c r="AB3" t="inlineStr">
         <is>
-          <t>669902430384160770-10299141-0-0-0-0-0-0</t>
+          <t>667755455610748930-10294535-0-0-0-0-0-0</t>
         </is>
       </c>
       <c r="AC3" t="n">
         <v>0</v>
       </c>
       <c r="AD3" t="inlineStr"/>
-      <c r="AE3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG3" t="inlineStr">
-        <is>
-          <t>https://cdn.staticsoe.com/pics/c3c82240030121c3097885c7797868d016c109819302bd20f74d67efc3c32bd1.jpg</t>
-        </is>
-      </c>
-      <c r="AH3" t="inlineStr"/>
-      <c r="AI3" t="inlineStr"/>
-      <c r="AJ3" t="inlineStr"/>
-      <c r="AK3" t="inlineStr"/>
+      <c r="AE3" t="inlineStr"/>
+      <c r="AF3" t="inlineStr"/>
+      <c r="AG3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH3" t="inlineStr">
+        <is>
+          <t>https://cdn.staticsoe.com/pics/84015f5c1ac3981cd391c1ebbac3e0dc9b1f5d9c3c50fec47b715bb2fd3841ff.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
         <v>10299140</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>2026-06-23T13:52:11-05:00</t>
-        </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -1014,34 +970,24 @@
         <v>0</v>
       </c>
       <c r="AD4" t="inlineStr"/>
-      <c r="AE4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG4" t="inlineStr">
+      <c r="AE4" t="inlineStr"/>
+      <c r="AF4" t="inlineStr"/>
+      <c r="AG4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH4" t="inlineStr">
         <is>
           <t>https://cdn.staticsoe.com/pics/84015f5c1ac3981cd391c1ebbac3e0dc9b1f5d9c3c50fec47b715bb2fd3841ff.jpg</t>
         </is>
       </c>
-      <c r="AH4" t="inlineStr"/>
-      <c r="AI4" t="inlineStr"/>
-      <c r="AJ4" t="inlineStr"/>
-      <c r="AK4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>10299139</v>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>2026-06-23T13:51:28-05:00</t>
-        </is>
+        <v>10294536</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>The Kinetic - Full Kit</t>
+          <t>The Kinetic</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -1052,38 +998,38 @@
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Ready-to-Play Full Kit — Jersey + Shorts</t>
+          <t>Ready-to-Play — Customize in seconds</t>
         </is>
       </c>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Electric motion lines built for speed. Complete matchday kit — jersey + matching shorts, fully customizable with your name and number.</t>
+          <t>Electric motion lines in purple, black &amp; cyan by default — recolor every zone, add your name and number, see it live.</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>{"type":"3d","mudel":"configId=mamuto316757&amp;suitName=mamuto3","activity":"","productId":"16757"}</t>
+          <t>{"type":"3d","mudel":"configId=mamuto316579&amp;suitName=mamuto3","activity":"","productId":"16579"}</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>The Kinetic Full Kit — Jersey + Shorts | MOMUTO</t>
+          <t>The Kinetic — Custom Football Jersey | MOMUTO</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>The Kinetic full kit — custom jersey + matching shorts in your colors, name and number, previewed live. Ready-to-Play, no minimum order.</t>
+          <t>Customize The Kinetic football jersey — your colors, name and number, previewed live. Ready-to-Play from €19.70. No minimum order, purchase-protected.</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>the-kinetic-full-kit</t>
+          <t>the-kinetic</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>custom football full kit, the kinetic jersey, momuto, ready to play kit, personalized soccer jersey, custom team kit, jersey and shorts, full football kit</t>
+          <t>custom football jersey, the kinetic jersey, momuto, ready to play kit, personalized soccer jersey, custom team kit</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -1098,7 +1044,7 @@
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>669902023787937794</t>
+          <t>667795838024155140</t>
         </is>
       </c>
       <c r="Q5" t="n">
@@ -1119,48 +1065,38 @@
       <c r="X5" t="inlineStr"/>
       <c r="Y5" t="inlineStr"/>
       <c r="Z5" t="n">
-        <v>51.1</v>
+        <v>35</v>
       </c>
       <c r="AA5" t="n">
         <v>0</v>
       </c>
       <c r="AB5" t="inlineStr">
         <is>
-          <t>669902023787937794-10299139-0-0-0-0-0-0</t>
+          <t>667795838024155140-10294536-0-0-0-0-0-0</t>
         </is>
       </c>
       <c r="AC5" t="n">
         <v>0</v>
       </c>
       <c r="AD5" t="inlineStr"/>
-      <c r="AE5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG5" t="inlineStr">
+      <c r="AE5" t="inlineStr"/>
+      <c r="AF5" t="inlineStr"/>
+      <c r="AG5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH5" t="inlineStr">
         <is>
           <t>https://cdn.staticsoe.com/pics/a1bcd4a78b3f3cdb245c9a37025dd5965760143c719ec3b77e1e7026af8bd1d1.jpg</t>
         </is>
       </c>
-      <c r="AH5" t="inlineStr"/>
-      <c r="AI5" t="inlineStr"/>
-      <c r="AJ5" t="inlineStr"/>
-      <c r="AK5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>10299138</v>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>2026-06-23T13:50:35-05:00</t>
-        </is>
+        <v>10299139</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>The Khala - Full Kit</t>
+          <t>The Kinetic - Full Kit</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -1177,32 +1113,32 @@
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Bold solid side panels and a fearless front. Complete matchday kit — jersey + matching shorts, fully customizable with your name and number.</t>
+          <t>Electric motion lines built for speed. Complete matchday kit — jersey + matching shorts, fully customizable with your name and number.</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>{"type":"3d","mudel":"configId=mamuto316756&amp;suitName=mamuto3","activity":"Shorts","productId":16756}</t>
+          <t>{"type":"3d","mudel":"configId=mamuto316757&amp;suitName=mamuto3","activity":"","productId":"16757"}</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>The Khala Full Kit — Jersey + Shorts | MOMUTO</t>
+          <t>The Kinetic Full Kit — Jersey + Shorts | MOMUTO</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>The Khala full kit — custom jersey + matching shorts in your colors, name and number, previewed live. Ready-to-Play, no minimum order.</t>
+          <t>The Kinetic full kit — custom jersey + matching shorts in your colors, name and number, previewed live. Ready-to-Play, no minimum order.</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>the-khala-full-kit</t>
+          <t>the-kinetic-full-kit</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>custom football full kit, the khala jersey, momuto, ready to play kit, personalized soccer jersey, custom team kit, jersey and shorts, full football kit</t>
+          <t>custom football full kit, the kinetic jersey, momuto, ready to play kit, personalized soccer jersey, custom team kit, jersey and shorts, full football kit</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -1217,7 +1153,7 @@
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>669901798902202371</t>
+          <t>669902023787937794</t>
         </is>
       </c>
       <c r="Q6" t="n">
@@ -1245,41 +1181,31 @@
       </c>
       <c r="AB6" t="inlineStr">
         <is>
-          <t>669901798902202371-10299138-0-0-0-0-0-0</t>
+          <t>669902023787937794-10299139-0-0-0-0-0-0</t>
         </is>
       </c>
       <c r="AC6" t="n">
         <v>0</v>
       </c>
       <c r="AD6" t="inlineStr"/>
-      <c r="AE6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG6" t="inlineStr">
-        <is>
-          <t>https://cdn.staticsoe.com/pics/a49782fe9cba8ef500eb9d4487d28b286fb027a09a1721a4f6d283feefc6bd8f.jpg</t>
-        </is>
-      </c>
-      <c r="AH6" t="inlineStr"/>
-      <c r="AI6" t="inlineStr"/>
-      <c r="AJ6" t="inlineStr"/>
-      <c r="AK6" t="inlineStr"/>
+      <c r="AE6" t="inlineStr"/>
+      <c r="AF6" t="inlineStr"/>
+      <c r="AG6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH6" t="inlineStr">
+        <is>
+          <t>https://cdn.staticsoe.com/pics/a1bcd4a78b3f3cdb245c9a37025dd5965760143c719ec3b77e1e7026af8bd1d1.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>10299137</v>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>2026-06-23T13:49:49-05:00</t>
-        </is>
+        <v>10299131</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>The Legacy - Full Kit</t>
+          <t>The Khala</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -1290,38 +1216,38 @@
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Ready-to-Play Full Kit — Jersey + Shorts</t>
+          <t>Ready-to-Play — Customize in seconds</t>
         </is>
       </c>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Heritage stripes, timeless by design. Complete matchday kit — jersey + matching shorts, fully customizable with your name and number.</t>
+          <t>Bold solid side panels and a striking front — fully recolorable to your club colors. Name and number included.</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>{"type":"3d","mudel":"configId=mamuto316755&amp;suitName=mamuto3","activity":"","productId":"16755"}</t>
+          <t>{"type":"3d","mudel":"configId=mamuto316678&amp;suitName=mamuto3","activity":"Shorts","productId":16678}</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>The Legacy Full Kit — Jersey + Shorts | MOMUTO</t>
+          <t>The Khala — Custom Football Jersey | MOMUTO</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>The Legacy full kit — custom jersey + matching shorts in your colors, name and number, previewed live. Ready-to-Play, no minimum order.</t>
+          <t>Customize The Khala football jersey — bold side panels in your club colors, name and number, previewed live. Ready-to-Play from €19.70. No minimum.</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>the-legacy-full-kit</t>
+          <t>the-khala</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>custom football full kit, the legacy jersey, momuto, ready to play kit, personalized soccer jersey, classic football kit, jersey and shorts, full football kit</t>
+          <t>custom football jersey, the khala jersey, momuto, ready to play kit, personalized soccer jersey, custom team kit</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -1336,7 +1262,7 @@
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>669901608586838016</t>
+          <t>669457844610531330</t>
         </is>
       </c>
       <c r="Q7" t="n">
@@ -1357,48 +1283,38 @@
       <c r="X7" t="inlineStr"/>
       <c r="Y7" t="inlineStr"/>
       <c r="Z7" t="n">
-        <v>51.1</v>
+        <v>35</v>
       </c>
       <c r="AA7" t="n">
         <v>0</v>
       </c>
       <c r="AB7" t="inlineStr">
         <is>
-          <t>669901608586838016-10299137-0-0-0-0-0-0</t>
+          <t>669457844610531330-10299131-0-0-0-0-0-0</t>
         </is>
       </c>
       <c r="AC7" t="n">
         <v>0</v>
       </c>
       <c r="AD7" t="inlineStr"/>
-      <c r="AE7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG7" t="inlineStr">
-        <is>
-          <t>https://cdn.staticsoe.com/pics/e62f0e8dbfcd718d2bfc043c6ca85645e8836aed76046dcf095dc6275e876050.jpg</t>
-        </is>
-      </c>
-      <c r="AH7" t="inlineStr"/>
-      <c r="AI7" t="inlineStr"/>
-      <c r="AJ7" t="inlineStr"/>
-      <c r="AK7" t="inlineStr"/>
+      <c r="AE7" t="inlineStr"/>
+      <c r="AF7" t="inlineStr"/>
+      <c r="AG7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH7" t="inlineStr">
+        <is>
+          <t>https://cdn.staticsoe.com/pics/368482b72b5c435b66cfbbabce8943e8ca57434ee5715699faf727aa36709d72.png</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>10299136</v>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>2026-06-23T13:49:08-05:00</t>
-        </is>
+        <v>10299138</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>The Mosaic - Full Kit</t>
+          <t>The Khala - Full Kit</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -1415,32 +1331,32 @@
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Tiled artwork you wear on the pitch. Complete matchday kit — jersey + matching shorts, fully customizable with your name and number.</t>
+          <t>Bold solid side panels and a fearless front. Complete matchday kit — jersey + matching shorts, fully customizable with your name and number.</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>{"type":"3d","mudel":"configId=mamuto316754&amp;suitName=mamuto3","activity":"","productId":"16754"}</t>
+          <t>{"type":"3d","mudel":"configId=mamuto316756&amp;suitName=mamuto3","activity":"Shorts","productId":16756}</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>The Mosaic Full Kit — Jersey + Shorts | MOMUTO</t>
+          <t>The Khala Full Kit — Jersey + Shorts | MOMUTO</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>The Mosaic full kit — custom jersey + matching shorts in your colors, name and number, previewed live. Ready-to-Play, no minimum order.</t>
+          <t>The Khala full kit — custom jersey + matching shorts in your colors, name and number, previewed live. Ready-to-Play, no minimum order.</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>the-mosaic-full-kit</t>
+          <t>the-khala-full-kit</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>custom football full kit, the mosaic jersey, momuto, ready to play kit, personalized soccer jersey, patterned football kit, jersey and shorts, full football kit</t>
+          <t>custom football full kit, the khala jersey, momuto, ready to play kit, personalized soccer jersey, custom team kit, jersey and shorts, full football kit</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -1455,7 +1371,7 @@
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>669901436660613120</t>
+          <t>669901798902202371</t>
         </is>
       </c>
       <c r="Q8" t="n">
@@ -1483,41 +1399,31 @@
       </c>
       <c r="AB8" t="inlineStr">
         <is>
-          <t>669901436660613120-10299136-0-0-0-0-0-0</t>
+          <t>669901798902202371-10299138-0-0-0-0-0-0</t>
         </is>
       </c>
       <c r="AC8" t="n">
         <v>0</v>
       </c>
       <c r="AD8" t="inlineStr"/>
-      <c r="AE8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG8" t="inlineStr">
-        <is>
-          <t>https://cdn.staticsoe.com/pics/84d0ff25a69c5a9f8f03b02a408daf54b5f356e49127849c727bfc0fc80e511f.jpg</t>
-        </is>
-      </c>
-      <c r="AH8" t="inlineStr"/>
-      <c r="AI8" t="inlineStr"/>
-      <c r="AJ8" t="inlineStr"/>
-      <c r="AK8" t="inlineStr"/>
+      <c r="AE8" t="inlineStr"/>
+      <c r="AF8" t="inlineStr"/>
+      <c r="AG8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH8" t="inlineStr">
+        <is>
+          <t>https://cdn.staticsoe.com/pics/a49782fe9cba8ef500eb9d4487d28b286fb027a09a1721a4f6d283feefc6bd8f.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>10299135</v>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>2026-06-23T13:48:14-05:00</t>
-        </is>
+        <v>10299132</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>The Prism - Full Kit</t>
+          <t>The Legacy</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1528,38 +1434,38 @@
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Ready-to-Play Full Kit — Jersey + Shorts</t>
+          <t>Ready-to-Play — Customize in seconds</t>
         </is>
       </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Faceted geometry — every angle counts. Complete matchday kit — jersey + matching shorts, fully customizable with your name and number.</t>
+          <t>Timeless heritage stripes in gold, navy &amp; green by default — recolor to your club, add your name and number.</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>{"type":"3d","mudel":"configId=mamuto316753&amp;suitName=mamuto3","activity":"Shorts","productId":16753}</t>
+          <t>{"type":"3d","mudel":"configId=mamuto316679&amp;suitName=mamuto3","activity":"Shorts","productId":16679}</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>The Prism Full Kit — Jersey + Shorts | MOMUTO</t>
+          <t>The Legacy — Custom Football Jersey | MOMUTO</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>The Prism full kit — custom jersey + matching shorts in your colors, name and number, previewed live. Ready-to-Play, no minimum order.</t>
+          <t>Customize The Legacy football jersey — timeless heritage stripes in your colors, name and number, previewed live. Ready-to-Play from €19.70.</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>the-prism-full-kit</t>
+          <t>the-legacy</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>custom football full kit, the prism jersey, momuto, ready to play kit, personalized soccer jersey, geometric football kit, jersey and shorts, full football kit</t>
+          <t>custom football jersey, the legacy jersey, momuto, ready to play kit, personalized soccer jersey, classic football kit</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1574,7 +1480,7 @@
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>669901209068503040</t>
+          <t>669458371986849792</t>
         </is>
       </c>
       <c r="Q9" t="n">
@@ -1595,48 +1501,38 @@
       <c r="X9" t="inlineStr"/>
       <c r="Y9" t="inlineStr"/>
       <c r="Z9" t="n">
-        <v>51.1</v>
+        <v>35</v>
       </c>
       <c r="AA9" t="n">
         <v>0</v>
       </c>
       <c r="AB9" t="inlineStr">
         <is>
-          <t>669901209068503040-10299135-0-0-0-0-0-0</t>
+          <t>669458371986849792-10299132-0-0-0-0-0-0</t>
         </is>
       </c>
       <c r="AC9" t="n">
         <v>0</v>
       </c>
       <c r="AD9" t="inlineStr"/>
-      <c r="AE9" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF9" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG9" t="inlineStr">
-        <is>
-          <t>https://cdn.staticsoe.com/pics/b0aa7df6e6789ef66b2c5032076007ad1d240440ff1192a6b043195fb0d9ff77.jpg</t>
-        </is>
-      </c>
-      <c r="AH9" t="inlineStr"/>
-      <c r="AI9" t="inlineStr"/>
-      <c r="AJ9" t="inlineStr"/>
-      <c r="AK9" t="inlineStr"/>
+      <c r="AE9" t="inlineStr"/>
+      <c r="AF9" t="inlineStr"/>
+      <c r="AG9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH9" t="inlineStr">
+        <is>
+          <t>https://cdn.staticsoe.com/pics/e62f0e8dbfcd718d2bfc043c6ca85645e8836aed76046dcf095dc6275e876050.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>10299134</v>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>2026-06-22T08:30:10-05:00</t>
-        </is>
+        <v>10299137</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>The Prism</t>
+          <t>The Legacy - Full Kit</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1647,38 +1543,38 @@
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Ready-to-Play — Customize in seconds</t>
+          <t>Ready-to-Play Full Kit — Jersey + Shorts</t>
         </is>
       </c>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Faceted geometric panels in maroon, grey &amp; green by default — recolor every zone, add your name and number, see it live.</t>
+          <t>Heritage stripes, timeless by design. Complete matchday kit — jersey + matching shorts, fully customizable with your name and number.</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>{"type":"3d","mudel":"configId=mamuto316681&amp;suitName=mamuto3","activity":"Shorts","productId":16681}</t>
+          <t>{"type":"3d","mudel":"configId=mamuto316755&amp;suitName=mamuto3","activity":"","productId":"16755"}</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>The Prism — Custom Football Jersey | MOMUTO</t>
+          <t>The Legacy Full Kit — Jersey + Shorts | MOMUTO</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>Customize The Prism football jersey — faceted geometric design in your colors, name and number, previewed live. Ready-to-Play from €19.70.</t>
+          <t>The Legacy full kit — custom jersey + matching shorts in your colors, name and number, previewed live. Ready-to-Play, no minimum order.</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>the-prism</t>
+          <t>the-legacy-full-kit</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>custom football jersey, the prism jersey, momuto, ready to play kit, personalized soccer jersey, geometric football kit</t>
+          <t>custom football full kit, the legacy jersey, momuto, ready to play kit, personalized soccer jersey, classic football kit, jersey and shorts, full football kit</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -1693,7 +1589,7 @@
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>669458779096743936</t>
+          <t>669901608586838016</t>
         </is>
       </c>
       <c r="Q10" t="n">
@@ -1714,44 +1610,34 @@
       <c r="X10" t="inlineStr"/>
       <c r="Y10" t="inlineStr"/>
       <c r="Z10" t="n">
-        <v>35</v>
+        <v>51.1</v>
       </c>
       <c r="AA10" t="n">
         <v>0</v>
       </c>
       <c r="AB10" t="inlineStr">
         <is>
-          <t>669458779096743936-10299134-0-0-0-0-0-0</t>
+          <t>669901608586838016-10299137-0-0-0-0-0-0</t>
         </is>
       </c>
       <c r="AC10" t="n">
         <v>0</v>
       </c>
       <c r="AD10" t="inlineStr"/>
-      <c r="AE10" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF10" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG10" t="inlineStr">
-        <is>
-          <t>https://cdn.staticsoe.com/pics/b0aa7df6e6789ef66b2c5032076007ad1d240440ff1192a6b043195fb0d9ff77.jpg</t>
-        </is>
-      </c>
-      <c r="AH10" t="inlineStr"/>
-      <c r="AI10" t="inlineStr"/>
-      <c r="AJ10" t="inlineStr"/>
-      <c r="AK10" t="inlineStr"/>
+      <c r="AE10" t="inlineStr"/>
+      <c r="AF10" t="inlineStr"/>
+      <c r="AG10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH10" t="inlineStr">
+        <is>
+          <t>https://cdn.staticsoe.com/pics/e62f0e8dbfcd718d2bfc043c6ca85645e8836aed76046dcf095dc6275e876050.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
         <v>10299133</v>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>2026-06-22T08:29:21-05:00</t>
-        </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -1847,34 +1733,24 @@
         <v>0</v>
       </c>
       <c r="AD11" t="inlineStr"/>
-      <c r="AE11" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF11" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG11" t="inlineStr">
+      <c r="AE11" t="inlineStr"/>
+      <c r="AF11" t="inlineStr"/>
+      <c r="AG11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH11" t="inlineStr">
         <is>
           <t>https://cdn.staticsoe.com/pics/84d0ff25a69c5a9f8f03b02a408daf54b5f356e49127849c727bfc0fc80e511f.jpg</t>
         </is>
       </c>
-      <c r="AH11" t="inlineStr"/>
-      <c r="AI11" t="inlineStr"/>
-      <c r="AJ11" t="inlineStr"/>
-      <c r="AK11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>10299132</v>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>2026-06-22T08:28:33-05:00</t>
-        </is>
+        <v>10299136</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>The Legacy</t>
+          <t>The Mosaic - Full Kit</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1885,38 +1761,38 @@
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Ready-to-Play — Customize in seconds</t>
+          <t>Ready-to-Play Full Kit — Jersey + Shorts</t>
         </is>
       </c>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Timeless heritage stripes in gold, navy &amp; green by default — recolor to your club, add your name and number.</t>
+          <t>Tiled artwork you wear on the pitch. Complete matchday kit — jersey + matching shorts, fully customizable with your name and number.</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>{"type":"3d","mudel":"configId=mamuto316679&amp;suitName=mamuto3","activity":"Shorts","productId":16679}</t>
+          <t>{"type":"3d","mudel":"configId=mamuto316754&amp;suitName=mamuto3","activity":"","productId":"16754"}</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>The Legacy — Custom Football Jersey | MOMUTO</t>
+          <t>The Mosaic Full Kit — Jersey + Shorts | MOMUTO</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>Customize The Legacy football jersey — timeless heritage stripes in your colors, name and number, previewed live. Ready-to-Play from €19.70.</t>
+          <t>The Mosaic full kit — custom jersey + matching shorts in your colors, name and number, previewed live. Ready-to-Play, no minimum order.</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>the-legacy</t>
+          <t>the-mosaic-full-kit</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>custom football jersey, the legacy jersey, momuto, ready to play kit, personalized soccer jersey, classic football kit</t>
+          <t>custom football full kit, the mosaic jersey, momuto, ready to play kit, personalized soccer jersey, patterned football kit, jersey and shorts, full football kit</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -1931,7 +1807,7 @@
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>669458371986849792</t>
+          <t>669901436660613120</t>
         </is>
       </c>
       <c r="Q12" t="n">
@@ -1952,48 +1828,38 @@
       <c r="X12" t="inlineStr"/>
       <c r="Y12" t="inlineStr"/>
       <c r="Z12" t="n">
-        <v>35</v>
+        <v>51.1</v>
       </c>
       <c r="AA12" t="n">
         <v>0</v>
       </c>
       <c r="AB12" t="inlineStr">
         <is>
-          <t>669458371986849792-10299132-0-0-0-0-0-0</t>
+          <t>669901436660613120-10299136-0-0-0-0-0-0</t>
         </is>
       </c>
       <c r="AC12" t="n">
         <v>0</v>
       </c>
       <c r="AD12" t="inlineStr"/>
-      <c r="AE12" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF12" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG12" t="inlineStr">
-        <is>
-          <t>https://cdn.staticsoe.com/pics/e62f0e8dbfcd718d2bfc043c6ca85645e8836aed76046dcf095dc6275e876050.jpg</t>
-        </is>
-      </c>
-      <c r="AH12" t="inlineStr"/>
-      <c r="AI12" t="inlineStr"/>
-      <c r="AJ12" t="inlineStr"/>
-      <c r="AK12" t="inlineStr"/>
+      <c r="AE12" t="inlineStr"/>
+      <c r="AF12" t="inlineStr"/>
+      <c r="AG12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH12" t="inlineStr">
+        <is>
+          <t>https://cdn.staticsoe.com/pics/84d0ff25a69c5a9f8f03b02a408daf54b5f356e49127849c727bfc0fc80e511f.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>10299131</v>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>2026-06-22T08:26:28-05:00</t>
-        </is>
+        <v>10299134</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>The Khala</t>
+          <t>The Prism</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -2010,32 +1876,32 @@
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Bold solid side panels and a striking front — fully recolorable to your club colors. Name and number included.</t>
+          <t>Faceted geometric panels in maroon, grey &amp; green by default — recolor every zone, add your name and number, see it live.</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>{"type":"3d","mudel":"configId=mamuto316678&amp;suitName=mamuto3","activity":"Shorts","productId":16678}</t>
+          <t>{"type":"3d","mudel":"configId=mamuto316681&amp;suitName=mamuto3","activity":"Shorts","productId":16681}</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>The Khala — Custom Football Jersey | MOMUTO</t>
+          <t>The Prism — Custom Football Jersey | MOMUTO</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>Customize The Khala football jersey — bold side panels in your club colors, name and number, previewed live. Ready-to-Play from €19.70. No minimum.</t>
+          <t>Customize The Prism football jersey — faceted geometric design in your colors, name and number, previewed live. Ready-to-Play from €19.70.</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>the-khala</t>
+          <t>the-prism</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>custom football jersey, the khala jersey, momuto, ready to play kit, personalized soccer jersey, custom team kit</t>
+          <t>custom football jersey, the prism jersey, momuto, ready to play kit, personalized soccer jersey, geometric football kit</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -2050,7 +1916,7 @@
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>669457844610531330</t>
+          <t>669458779096743936</t>
         </is>
       </c>
       <c r="Q13" t="n">
@@ -2078,41 +1944,31 @@
       </c>
       <c r="AB13" t="inlineStr">
         <is>
-          <t>669457844610531330-10299131-0-0-0-0-0-0</t>
+          <t>669458779096743936-10299134-0-0-0-0-0-0</t>
         </is>
       </c>
       <c r="AC13" t="n">
         <v>0</v>
       </c>
       <c r="AD13" t="inlineStr"/>
-      <c r="AE13" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF13" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG13" t="inlineStr">
-        <is>
-          <t>https://cdn.staticsoe.com/pics/368482b72b5c435b66cfbbabce8943e8ca57434ee5715699faf727aa36709d72.png</t>
-        </is>
-      </c>
-      <c r="AH13" t="inlineStr"/>
-      <c r="AI13" t="inlineStr"/>
-      <c r="AJ13" t="inlineStr"/>
-      <c r="AK13" t="inlineStr"/>
+      <c r="AE13" t="inlineStr"/>
+      <c r="AF13" t="inlineStr"/>
+      <c r="AG13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH13" t="inlineStr">
+        <is>
+          <t>https://cdn.staticsoe.com/pics/b0aa7df6e6789ef66b2c5032076007ad1d240440ff1192a6b043195fb0d9ff77.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>10294536</v>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>2026-06-17T18:22:14-05:00</t>
-        </is>
+        <v>10299135</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>The Kinetic</t>
+          <t>The Prism - Full Kit</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -2123,38 +1979,38 @@
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Ready-to-Play — Customize in seconds</t>
+          <t>Ready-to-Play Full Kit — Jersey + Shorts</t>
         </is>
       </c>
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Electric motion lines in purple, black &amp; cyan by default — recolor every zone, add your name and number, see it live.</t>
+          <t>Faceted geometry — every angle counts. Complete matchday kit — jersey + matching shorts, fully customizable with your name and number.</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>{"type":"3d","mudel":"configId=mamuto316579&amp;suitName=mamuto3","activity":"","productId":"16579"}</t>
+          <t>{"type":"3d","mudel":"configId=mamuto316753&amp;suitName=mamuto3","activity":"Shorts","productId":16753}</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>The Kinetic — Custom Football Jersey | MOMUTO</t>
+          <t>The Prism Full Kit — Jersey + Shorts | MOMUTO</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>Customize The Kinetic football jersey — your colors, name and number, previewed live. Ready-to-Play from €19.70. No minimum order, purchase-protected.</t>
+          <t>The Prism full kit — custom jersey + matching shorts in your colors, name and number, previewed live. Ready-to-Play, no minimum order.</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>the-kinetic</t>
+          <t>the-prism-full-kit</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>custom football jersey, the kinetic jersey, momuto, ready to play kit, personalized soccer jersey, custom team kit</t>
+          <t>custom football full kit, the prism jersey, momuto, ready to play kit, personalized soccer jersey, geometric football kit, jersey and shorts, full football kit</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
@@ -2169,7 +2025,7 @@
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>667795838024155140</t>
+          <t>669901209068503040</t>
         </is>
       </c>
       <c r="Q14" t="n">
@@ -2190,48 +2046,38 @@
       <c r="X14" t="inlineStr"/>
       <c r="Y14" t="inlineStr"/>
       <c r="Z14" t="n">
-        <v>35</v>
+        <v>51.1</v>
       </c>
       <c r="AA14" t="n">
         <v>0</v>
       </c>
       <c r="AB14" t="inlineStr">
         <is>
-          <t>667795838024155140-10294536-0-0-0-0-0-0</t>
+          <t>669901209068503040-10299135-0-0-0-0-0-0</t>
         </is>
       </c>
       <c r="AC14" t="n">
         <v>0</v>
       </c>
       <c r="AD14" t="inlineStr"/>
-      <c r="AE14" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF14" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG14" t="inlineStr">
-        <is>
-          <t>https://cdn.staticsoe.com/pics/a1bcd4a78b3f3cdb245c9a37025dd5965760143c719ec3b77e1e7026af8bd1d1.jpg</t>
-        </is>
-      </c>
-      <c r="AH14" t="inlineStr"/>
-      <c r="AI14" t="inlineStr"/>
-      <c r="AJ14" t="inlineStr"/>
-      <c r="AK14" t="inlineStr"/>
+      <c r="AE14" t="inlineStr"/>
+      <c r="AF14" t="inlineStr"/>
+      <c r="AG14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH14" t="inlineStr">
+        <is>
+          <t>https://cdn.staticsoe.com/pics/b0aa7df6e6789ef66b2c5032076007ad1d240440ff1192a6b043195fb0d9ff77.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>10294535</v>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>2026-06-17T15:41:46-05:00</t>
-        </is>
+        <v>10294534</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>The Apex</t>
+          <t>The Fracture</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -2248,32 +2094,32 @@
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Bold angular shoulder panels in navy &amp; volt by default — fully recolorable. Add your name and number and play this week.</t>
+          <t>A striking angular shard pattern — fully recolorable to your club. Add your name and number and play this week.</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>{"type":"3d","mudel":"configId=mamuto316578&amp;suitName=mamuto3","activity":"","productId":"16578"}</t>
+          <t>{"type":"3d","mudel":"configId=mamuto316534&amp;suitName=mamuto3","activity":"","productId":"16534"}</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>The Apex — Custom Football Jersey | MOMUTO</t>
+          <t>The Fracture — Custom Football Jersey | MOMUTO</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>Customize The Apex football jersey — your colors, name and number, previewed live. Ready-to-Play from €19.70. No minimum order, every order purchase-protected.</t>
+          <t>Customize The Fracture football jersey — striking angular shard design in your colors, name and number, previewed live. Ready-to-Play from €19.70.</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>the-apex</t>
+          <t>the-fracture</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>custom football jersey, the apex jersey, momuto, ready to play kit, personalized soccer jersey, custom team kit</t>
+          <t>custom football jersey, the fracture jersey, momuto, ready to play kit, personalized soccer jersey, modern football kit</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
@@ -2288,7 +2134,7 @@
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>667755455610748930</t>
+          <t>667275927320526848</t>
         </is>
       </c>
       <c r="Q15" t="n">
@@ -2316,41 +2162,31 @@
       </c>
       <c r="AB15" t="inlineStr">
         <is>
-          <t>667755455610748930-10294535-0-0-0-0-0-0</t>
+          <t>667275927320526848-10294534-0-0-0-0-0-0</t>
         </is>
       </c>
       <c r="AC15" t="n">
         <v>0</v>
       </c>
       <c r="AD15" t="inlineStr"/>
-      <c r="AE15" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF15" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG15" t="inlineStr">
-        <is>
-          <t>https://cdn.staticsoe.com/pics/84015f5c1ac3981cd391c1ebbac3e0dc9b1f5d9c3c50fec47b715bb2fd3841ff.jpg</t>
-        </is>
-      </c>
-      <c r="AH15" t="inlineStr"/>
-      <c r="AI15" t="inlineStr"/>
-      <c r="AJ15" t="inlineStr"/>
-      <c r="AK15" t="inlineStr"/>
+      <c r="AE15" t="inlineStr"/>
+      <c r="AF15" t="inlineStr"/>
+      <c r="AG15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH15" t="inlineStr">
+        <is>
+          <t>https://cdn.staticsoe.com/pics/c3c82240030121c3097885c7797868d016c109819302bd20f74d67efc3c32bd1.jpg,https://cdn.staticsoe.com/pics/6e1255435fceb296065f6bcb8f3e1f2a8198943d67808c2ff67078ec0b49eb92.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>10294534</v>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>2026-06-16T07:56:18-05:00</t>
-        </is>
+        <v>10299141</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>The Fracture</t>
+          <t>The Fracture - Full Kit</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -2361,38 +2197,38 @@
       <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Ready-to-Play — Customize in seconds</t>
+          <t>Ready-to-Play Full Kit — Jersey + Shorts</t>
         </is>
       </c>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr">
         <is>
-          <t>A striking angular shard pattern — fully recolorable to your club. Add your name and number and play this week.</t>
+          <t>Angular shards that break the standard. Complete matchday kit — jersey + matching shorts, fully customizable with your name and number.</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>{"type":"3d","mudel":"configId=mamuto316534&amp;suitName=mamuto3","activity":"","productId":"16534"}</t>
+          <t>{"type":"3d","mudel":"configId=mamuto316759&amp;suitName=mamuto3","activity":"","productId":"16759"}</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>The Fracture — Custom Football Jersey | MOMUTO</t>
+          <t>The Fracture Full Kit — Jersey + Shorts | MOMUTO</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>Customize The Fracture football jersey — striking angular shard design in your colors, name and number, previewed live. Ready-to-Play from €19.70.</t>
+          <t>The Fracture full kit — custom jersey + matching shorts in your colors, name and number, previewed live. Ready-to-Play, no minimum order.</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>the-fracture</t>
+          <t>the-fracture-full-kit</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>custom football jersey, the fracture jersey, momuto, ready to play kit, personalized soccer jersey, modern football kit</t>
+          <t>custom football full kit, the fracture jersey, momuto, ready to play kit, personalized soccer jersey, modern football kit, jersey and shorts, full football kit</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
@@ -2407,7 +2243,7 @@
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>667275927320526848</t>
+          <t>669902430384160770</t>
         </is>
       </c>
       <c r="Q16" t="n">
@@ -2428,39 +2264,30 @@
       <c r="X16" t="inlineStr"/>
       <c r="Y16" t="inlineStr"/>
       <c r="Z16" t="n">
-        <v>35</v>
+        <v>51.1</v>
       </c>
       <c r="AA16" t="n">
         <v>0</v>
       </c>
       <c r="AB16" t="inlineStr">
         <is>
-          <t>667275927320526848-10294534-0-0-0-0-0-0</t>
+          <t>669902430384160770-10299141-0-0-0-0-0-0</t>
         </is>
       </c>
       <c r="AC16" t="n">
         <v>0</v>
       </c>
       <c r="AD16" t="inlineStr"/>
-      <c r="AE16" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF16" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG16" t="inlineStr">
-        <is>
-          <t>https://cdn.staticsoe.com/pics/c3c82240030121c3097885c7797868d016c109819302bd20f74d67efc3c32bd1.jpg,https://cdn.staticsoe.com/pics/6e1255435fceb296065f6bcb8f3e1f2a8198943d67808c2ff67078ec0b49eb92.jpg</t>
-        </is>
+      <c r="AE16" t="inlineStr"/>
+      <c r="AF16" t="inlineStr"/>
+      <c r="AG16" t="n">
+        <v>0</v>
       </c>
       <c r="AH16" t="inlineStr">
         <is>
-          <t>|</t>
-        </is>
-      </c>
-      <c r="AI16" t="inlineStr"/>
-      <c r="AJ16" t="inlineStr"/>
-      <c r="AK16" t="inlineStr"/>
+          <t>https://cdn.staticsoe.com/pics/c3c82240030121c3097885c7797868d016c109819302bd20f74d67efc3c32bd1.jpg</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>